<commit_message>
GitHub araştırması 2. tur: gerçek MTY blokları (INSERT+öznitelik), kombi pompa/genleşme/kangal hesabı, psikrometri, BPDF uyumlu pafta sınırları, AutoCAD LISP araçları
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/sinem_turhan/SINEM_TURHAN_ISI_KAYBI_YERDEN_ISITMA_HIDROFOR.xlsx
+++ b/proje/sinem_turhan/SINEM_TURHAN_ISI_KAYBI_YERDEN_ISITMA_HIDROFOR.xlsx
@@ -18,9 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YERDEN ISITMA- DEVAMI" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HİDROFOR-POMPA" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YAĞMUR SUYU" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KOMBİ-POMPA-GENLEŞME" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'TEKNİK RAPOR'!$A$1:$N$65</definedName>
@@ -33,6 +34,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="8">'YERDEN ISITMA- DEVAMI'!$A$1:$AA$47</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'HİDROFOR-POMPA'!$A$1:$D$36</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'YAĞMUR SUYU'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'KOMBİ-POMPA-GENLEŞME'!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
@@ -879,7 +881,7 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="587">
+  <cellXfs count="589">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2644,6 +2646,12 @@
     </xf>
     <xf numFmtId="0" fontId="57" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="7" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -4643,6 +4651,367 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="244" min="1" max="1"/>
+    <col width="10" customWidth="1" style="244" min="2" max="2"/>
+    <col width="10" customWidth="1" style="244" min="3" max="3"/>
+    <col width="11" customWidth="1" style="244" min="4" max="4"/>
+    <col width="9" customWidth="1" style="244" min="5" max="5"/>
+    <col width="12" customWidth="1" style="244" min="6" max="6"/>
+    <col width="12" customWidth="1" style="244" min="7" max="7"/>
+    <col width="11" customWidth="1" style="244" min="8" max="8"/>
+    <col width="8" customWidth="1" style="244" min="9" max="9"/>
+    <col width="11" customWidth="1" style="244" min="10" max="10"/>
+    <col width="9" customWidth="1" style="244" min="11" max="11"/>
+    <col width="14" customWidth="1" style="244" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="580" t="inlineStr">
+        <is>
+          <t>KOMBİ POMPASI, GENLEŞME TANKI VE PEX KANGAL KONTROLÜ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="581" t="inlineStr">
+        <is>
+          <t>Pompa: H = Δp(en uzun devre, Churchill, yerel kayıp x1,3) + kollektör 5 kPa ;  Genleşme: Vmin = (P2+1,013)/(P2-P1) x (0,01 V + ΔV) , 10→50 °C</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="582" t="inlineStr">
+        <is>
+          <t>PROJE : SİNEM TURHAN'A AİT 3 BAĞIMSIZ BÖLÜMLÜ MESKEN (SERDİVAN 13748 PARSEL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="582" t="inlineStr">
+        <is>
+          <t>ROTAŞ MÜHENDİSLİK - Mak. Müh. Bayram GENÇ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="587" t="inlineStr">
+        <is>
+          <t>DAİRE</t>
+        </is>
+      </c>
+      <c r="B6" s="587" t="inlineStr">
+        <is>
+          <t>YÜK (W)</t>
+        </is>
+      </c>
+      <c r="C6" s="587" t="inlineStr">
+        <is>
+          <t>DEBİ (l/h)</t>
+        </is>
+      </c>
+      <c r="D6" s="587" t="inlineStr">
+        <is>
+          <t>Δp maks (kPa)</t>
+        </is>
+      </c>
+      <c r="E6" s="587" t="inlineStr">
+        <is>
+          <t>H (kPa)</t>
+        </is>
+      </c>
+      <c r="F6" s="587" t="inlineStr">
+        <is>
+          <t>Kombi pompası (kPa)</t>
+        </is>
+      </c>
+      <c r="G6" s="587" t="inlineStr">
+        <is>
+          <t>POMPA</t>
+        </is>
+      </c>
+      <c r="H6" s="587" t="inlineStr">
+        <is>
+          <t>Sistem suyu (l)</t>
+        </is>
+      </c>
+      <c r="I6" s="587" t="inlineStr">
+        <is>
+          <t>ΔV (l)</t>
+        </is>
+      </c>
+      <c r="J6" s="587" t="inlineStr">
+        <is>
+          <t>P1 / P2 (bar)</t>
+        </is>
+      </c>
+      <c r="K6" s="587" t="inlineStr">
+        <is>
+          <t>Vmin (l)</t>
+        </is>
+      </c>
+      <c r="L6" s="587" t="inlineStr">
+        <is>
+          <t>TANK (kombi 8 l)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="586" t="inlineStr">
+        <is>
+          <t>BODRUM DAİRE 1</t>
+        </is>
+      </c>
+      <c r="B7" s="586" t="n">
+        <v>4222</v>
+      </c>
+      <c r="C7" s="586" t="n">
+        <v>363</v>
+      </c>
+      <c r="D7" s="585" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E7" s="585">
+        <f>D7+5</f>
+        <v/>
+      </c>
+      <c r="F7" s="586" t="n">
+        <v>25</v>
+      </c>
+      <c r="G7" s="586">
+        <f>IF(E7&lt;=F7,"UYGUN","POMPA GRUBU")</f>
+        <v/>
+      </c>
+      <c r="H7" s="586" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="I7" s="585" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J7" s="586" t="inlineStr">
+        <is>
+          <t>0.5 / 2.5</t>
+        </is>
+      </c>
+      <c r="K7" s="585">
+        <f>(2.5+1.013)/(2.5-0.5)*(0.01*H7+I7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="586">
+        <f>IF(K7&lt;=8,"YETERLİ","İLAVE TANK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="586" t="inlineStr">
+        <is>
+          <t>ZEMİN DAİRE 2</t>
+        </is>
+      </c>
+      <c r="B8" s="586" t="n">
+        <v>3791</v>
+      </c>
+      <c r="C8" s="586" t="n">
+        <v>326</v>
+      </c>
+      <c r="D8" s="585" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E8" s="585">
+        <f>D8+5</f>
+        <v/>
+      </c>
+      <c r="F8" s="586" t="n">
+        <v>25</v>
+      </c>
+      <c r="G8" s="586">
+        <f>IF(E8&lt;=F8,"UYGUN","POMPA GRUBU")</f>
+        <v/>
+      </c>
+      <c r="H8" s="586" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="I8" s="585" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J8" s="586" t="inlineStr">
+        <is>
+          <t>0.5 / 2.5</t>
+        </is>
+      </c>
+      <c r="K8" s="585">
+        <f>(2.5+1.013)/(2.5-0.5)*(0.01*H8+I8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="586">
+        <f>IF(K8&lt;=8,"YETERLİ","İLAVE TANK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="586" t="inlineStr">
+        <is>
+          <t>1 NK DAİRE 3</t>
+        </is>
+      </c>
+      <c r="B9" s="586" t="n">
+        <v>4302</v>
+      </c>
+      <c r="C9" s="586" t="n">
+        <v>370</v>
+      </c>
+      <c r="D9" s="585" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="E9" s="585">
+        <f>D9+5</f>
+        <v/>
+      </c>
+      <c r="F9" s="586" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" s="586">
+        <f>IF(E9&lt;=F9,"UYGUN","POMPA GRUBU")</f>
+        <v/>
+      </c>
+      <c r="H9" s="586" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="I9" s="585" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J9" s="586" t="inlineStr">
+        <is>
+          <t>0.5 / 2.5</t>
+        </is>
+      </c>
+      <c r="K9" s="585">
+        <f>(2.5+1.013)/(2.5-0.5)*(0.01*H9+I9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="586">
+        <f>IF(K9&lt;=8,"YETERLİ","İLAVE TANK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="588" t="inlineStr">
+        <is>
+          <t>PEX 16x2,0 KANGAL METRAJI (devre ortasında ek yapılmaz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="587" t="inlineStr">
+        <is>
+          <t>DAİRE</t>
+        </is>
+      </c>
+      <c r="B12" s="587" t="inlineStr">
+        <is>
+          <t>TOPLAM (m)</t>
+        </is>
+      </c>
+      <c r="C12" s="587" t="inlineStr">
+        <is>
+          <t>200 m kangal</t>
+        </is>
+      </c>
+      <c r="D12" s="587" t="inlineStr">
+        <is>
+          <t>500 m kangal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="586" t="inlineStr">
+        <is>
+          <t>BODRUM DAİRE 1</t>
+        </is>
+      </c>
+      <c r="B13" s="586" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="C13" s="586" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="586" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="586" t="inlineStr">
+        <is>
+          <t>ZEMİN DAİRE 2</t>
+        </is>
+      </c>
+      <c r="B14" s="586" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="C14" s="586" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="586" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="586" t="inlineStr">
+        <is>
+          <t>1 NK DAİRE 3</t>
+        </is>
+      </c>
+      <c r="B15" s="586" t="n">
+        <v>558.8</v>
+      </c>
+      <c r="C15" s="586" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="586" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="582" t="inlineStr">
+        <is>
+          <t>Kombi pompasının kullanılabilir basma yüksekliği (25 kPa) seçilen kombinin kataloğundan teyit edilecektir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="582" t="inlineStr">
+        <is>
+          <t>Kombi içi genleşme tankı 8 l, emniyet ventili 3 bar, ilk dolum basıncı 1,0-1,5 bar alınmıştır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="582" t="inlineStr">
+        <is>
+          <t>Devre debileri kollektördeki debimetreli reglaj vanaları ile ayarlanacaktır.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>

<commit_message>
Excel: şablondaki dcm makina logosu tüm hesap dosyalarından kaldırıldı (logo_temizle)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/sinem_turhan/SINEM_TURHAN_ISI_KAYBI_YERDEN_ISITMA_HIDROFOR.xlsx
+++ b/proje/sinem_turhan/SINEM_TURHAN_ISI_KAYBI_YERDEN_ISITMA_HIDROFOR.xlsx
@@ -3088,141 +3088,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>261360</colOff>
-      <row>1</row>
-      <rowOff>37800</rowOff>
-    </from>
-    <to>
-      <col>0</col>
-      <colOff>1379880</colOff>
-      <row>5</row>
-      <rowOff>9360</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="0" name="Resim 1" descr=""/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="261360" y="247320"/>
-          <a:ext cx="1118520" cy="1200240"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>62280</colOff>
-      <row>3</row>
-      <rowOff>142920</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Resim 1" descr=""/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="443880" cy="476280"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>0</col>
-      <colOff>442800</colOff>
-      <row>2</row>
-      <rowOff>152640</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Resim 1" descr=""/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="442800" cy="476640"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -3944,7 +3809,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.157638888888889" right="0.157638888888889" top="0.479861111111111" bottom="0.157638888888889" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -21747,7 +21611,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -24642,7 +24505,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>